<commit_message>
Update data curation + add Waukee
</commit_message>
<xml_diff>
--- a/Scout/ankeny-centennial-vs-sep-082826.xlsx
+++ b/Scout/ankeny-centennial-vs-sep-082826.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <workbookPr defaultThemeVersion="202300"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1abc75c8e08b2b2b/Desktop/GitHub/Dowling-Football/Scout/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_2C88D02D490A992410231BC97880160831049C5E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC64045D-3E67-4811-9BEE-BD91CFA66E6D}"/>
   <bookViews>
-    <workbookView/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="Rddb5453876094615"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="0" uniqueCount="0">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1146" uniqueCount="86">
   <si>
     <t>PLAY #</t>
   </si>
@@ -273,11 +282,869 @@
 </sst>
 </file>
 
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="18" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Aptos Display"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="33">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+  </fills>
+  <borders count="10">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="42">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="42">
+    <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Note" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Title" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="0E2841"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E8E8E8"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="156082"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="E97132"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="196B24"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="0F9ED5"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="A02B93"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="4EA72E"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="467886"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="96607D"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
+  <a:extLst>
+    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+    </a:ext>
+  </a:extLst>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AC145"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="8" max="8" width="12.36328125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -366,7 +1233,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -389,7 +1256,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -439,7 +1306,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -489,7 +1356,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -539,7 +1406,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -592,7 +1459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -642,7 +1509,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -695,7 +1562,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -745,7 +1612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -795,7 +1662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -836,7 +1703,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -877,7 +1744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -903,7 +1770,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -926,7 +1793,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -973,7 +1840,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1023,7 +1890,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1070,7 +1937,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1120,7 +1987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1170,7 +2037,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1223,7 +2090,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1273,7 +2140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1323,7 +2190,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1373,7 +2240,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1423,7 +2290,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1446,7 +2313,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1496,7 +2363,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1549,7 +2416,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1599,7 +2466,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1649,7 +2516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1696,7 +2563,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1746,7 +2613,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1799,7 +2666,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1840,7 +2707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1890,7 +2757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1922,7 +2789,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1972,7 +2839,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1998,7 +2865,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2021,7 +2888,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2071,7 +2938,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>39</v>
       </c>
@@ -2121,7 +2988,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2171,7 +3038,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2221,7 +3088,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2274,7 +3141,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2321,7 +3188,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2371,7 +3238,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2421,7 +3288,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2471,7 +3338,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2497,7 +3364,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2523,7 +3390,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2573,7 +3440,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2623,7 +3490,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>51</v>
       </c>
@@ -2673,7 +3540,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>52</v>
       </c>
@@ -2705,7 +3572,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>53</v>
       </c>
@@ -2728,7 +3595,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>54</v>
       </c>
@@ -2781,7 +3648,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>55</v>
       </c>
@@ -2831,7 +3698,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>56</v>
       </c>
@@ -2881,7 +3748,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>57</v>
       </c>
@@ -2931,7 +3798,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>58</v>
       </c>
@@ -2981,7 +3848,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>59</v>
       </c>
@@ -3031,7 +3898,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>60</v>
       </c>
@@ -3081,7 +3948,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>61</v>
       </c>
@@ -3107,7 +3974,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>62</v>
       </c>
@@ -3130,7 +3997,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>63</v>
       </c>
@@ -3180,7 +4047,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>64</v>
       </c>
@@ -3230,7 +4097,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>65</v>
       </c>
@@ -3280,7 +4147,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>66</v>
       </c>
@@ -3330,7 +4197,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>67</v>
       </c>
@@ -3380,7 +4247,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>68</v>
       </c>
@@ -3412,7 +4279,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>69</v>
       </c>
@@ -3435,7 +4302,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>70</v>
       </c>
@@ -3446,7 +4313,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>71</v>
       </c>
@@ -3469,7 +4336,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>72</v>
       </c>
@@ -3519,7 +4386,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>73</v>
       </c>
@@ -3572,7 +4439,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>74</v>
       </c>
@@ -3622,7 +4489,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>75</v>
       </c>
@@ -3672,7 +4539,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>76</v>
       </c>
@@ -3722,7 +4589,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="78">
+    <row r="78" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>77</v>
       </c>
@@ -3748,7 +4615,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>78</v>
       </c>
@@ -3771,7 +4638,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>79</v>
       </c>
@@ -3821,7 +4688,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>80</v>
       </c>
@@ -3874,7 +4741,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>81</v>
       </c>
@@ -3924,7 +4791,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>82</v>
       </c>
@@ -3956,7 +4823,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>83</v>
       </c>
@@ -4006,7 +4873,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>84</v>
       </c>
@@ -4056,7 +4923,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="86">
+    <row r="86" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>85</v>
       </c>
@@ -4106,7 +4973,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>86</v>
       </c>
@@ -4138,7 +5005,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="88">
+    <row r="88" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>87</v>
       </c>
@@ -4191,7 +5058,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="89">
+    <row r="89" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>88</v>
       </c>
@@ -4238,7 +5105,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="90">
+    <row r="90" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>89</v>
       </c>
@@ -4291,7 +5158,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="91">
+    <row r="91" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>90</v>
       </c>
@@ -4341,7 +5208,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="92">
+    <row r="92" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>91</v>
       </c>
@@ -4373,7 +5240,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="93">
+    <row r="93" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>92</v>
       </c>
@@ -4423,7 +5290,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="94">
+    <row r="94" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>93</v>
       </c>
@@ -4473,7 +5340,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="95">
+    <row r="95" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>94</v>
       </c>
@@ -4496,7 +5363,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="96">
+    <row r="96" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>95</v>
       </c>
@@ -4546,7 +5413,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="97">
+    <row r="97" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>96</v>
       </c>
@@ -4587,7 +5454,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="98">
+    <row r="98" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>97</v>
       </c>
@@ -4637,7 +5504,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="99">
+    <row r="99" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>98</v>
       </c>
@@ -4687,7 +5554,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="100">
+    <row r="100" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>99</v>
       </c>
@@ -4737,7 +5604,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="101">
+    <row r="101" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>100</v>
       </c>
@@ -4787,7 +5654,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="102">
+    <row r="102" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A102">
         <v>101</v>
       </c>
@@ -4813,7 +5680,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="103">
+    <row r="103" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>102</v>
       </c>
@@ -4836,7 +5703,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="104">
+    <row r="104" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>103</v>
       </c>
@@ -4886,7 +5753,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="105">
+    <row r="105" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A105">
         <v>104</v>
       </c>
@@ -4936,7 +5803,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="106">
+    <row r="106" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>105</v>
       </c>
@@ -4986,7 +5853,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="107">
+    <row r="107" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A107">
         <v>106</v>
       </c>
@@ -5036,7 +5903,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="108">
+    <row r="108" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A108">
         <v>107</v>
       </c>
@@ -5086,7 +5953,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="109">
+    <row r="109" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A109">
         <v>108</v>
       </c>
@@ -5136,7 +6003,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="110">
+    <row r="110" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A110">
         <v>109</v>
       </c>
@@ -5186,7 +6053,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="111">
+    <row r="111" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A111">
         <v>110</v>
       </c>
@@ -5236,7 +6103,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="112">
+    <row r="112" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A112">
         <v>111</v>
       </c>
@@ -5286,7 +6153,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="113">
+    <row r="113" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A113">
         <v>112</v>
       </c>
@@ -5336,7 +6203,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="114">
+    <row r="114" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A114">
         <v>113</v>
       </c>
@@ -5386,7 +6253,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="115">
+    <row r="115" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A115">
         <v>114</v>
       </c>
@@ -5436,7 +6303,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="116">
+    <row r="116" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>115</v>
       </c>
@@ -5468,7 +6335,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="117">
+    <row r="117" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>116</v>
       </c>
@@ -5515,7 +6382,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="118">
+    <row r="118" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>117</v>
       </c>
@@ -5565,7 +6432,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="119">
+    <row r="119" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>118</v>
       </c>
@@ -5615,7 +6482,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="120">
+    <row r="120" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>119</v>
       </c>
@@ -5665,7 +6532,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="121">
+    <row r="121" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>120</v>
       </c>
@@ -5715,7 +6582,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="122">
+    <row r="122" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>121</v>
       </c>
@@ -5738,7 +6605,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="123">
+    <row r="123" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A123">
         <v>122</v>
       </c>
@@ -5779,7 +6646,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="124">
+    <row r="124" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>123</v>
       </c>
@@ -5829,7 +6696,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="125">
+    <row r="125" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>124</v>
       </c>
@@ -5882,7 +6749,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="126">
+    <row r="126" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>125</v>
       </c>
@@ -5923,7 +6790,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="127">
+    <row r="127" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A127">
         <v>126</v>
       </c>
@@ -5973,7 +6840,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="128">
+    <row r="128" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A128">
         <v>127</v>
       </c>
@@ -6005,7 +6872,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="129">
+    <row r="129" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A129">
         <v>128</v>
       </c>
@@ -6055,7 +6922,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="130">
+    <row r="130" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A130">
         <v>129</v>
       </c>
@@ -6105,7 +6972,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="131">
+    <row r="131" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A131">
         <v>130</v>
       </c>
@@ -6155,7 +7022,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="132">
+    <row r="132" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A132">
         <v>131</v>
       </c>
@@ -6205,7 +7072,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="133">
+    <row r="133" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A133">
         <v>132</v>
       </c>
@@ -6237,7 +7104,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="134">
+    <row r="134" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A134">
         <v>133</v>
       </c>
@@ -6287,7 +7154,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="135">
+    <row r="135" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A135">
         <v>134</v>
       </c>
@@ -6337,7 +7204,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="136">
+    <row r="136" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A136">
         <v>135</v>
       </c>
@@ -6387,7 +7254,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="137">
+    <row r="137" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A137">
         <v>136</v>
       </c>
@@ -6437,7 +7304,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="138">
+    <row r="138" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A138">
         <v>137</v>
       </c>
@@ -6487,7 +7354,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="139">
+    <row r="139" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A139">
         <v>138</v>
       </c>
@@ -6513,7 +7380,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="140">
+    <row r="140" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A140">
         <v>139</v>
       </c>
@@ -6536,7 +7403,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="141">
+    <row r="141" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A141">
         <v>140</v>
       </c>
@@ -6586,7 +7453,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="142">
+    <row r="142" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A142">
         <v>141</v>
       </c>
@@ -6636,7 +7503,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="143">
+    <row r="143" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A143">
         <v>142</v>
       </c>
@@ -6662,7 +7529,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="144">
+    <row r="144" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A144">
         <v>143</v>
       </c>
@@ -6685,7 +7552,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="145">
+    <row r="145" spans="1:28" x14ac:dyDescent="0.35">
       <c r="A145">
         <v>144</v>
       </c>
@@ -6736,5 +7603,6 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>